<commit_message>
commit message: "Refactor data reading and update test data sources
</commit_message>
<xml_diff>
--- a/test_data/loginData.xlsx
+++ b/test_data/loginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ridwa\OneDrive\Documents\Projects\Playwright\PlaywrightTSProject1\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E60FD3-7CFE-458E-A731-43052CAB9F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931A5225-6DF6-43F3-A0C3-FC2A7750ED74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -480,7 +480,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -494,13 +494,13 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:D3 A4:C4" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:D2 A4:C4 A3:C3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>